<commit_message>
Add Role-Based Access Control (Admin/Staff accounts)
Replaces the single shared TEAM_PASSWORD with real individual accounts
and two roles. Admin-only: deleting any record, editing a record someone
else created, and managing accounts from the new "Manage users" page.
A Staff member's History is scoped to documents they created; equipment
lookup, the register, and Resignation's list stay open to everyone since
they need cross-visibility to work.

Accounts are only ever created by an Admin, always with the same fixed
starting password, with a forced password-change screen before the
account can do anything else. Pre-existing records have no verified
owner until an Admin assigns one via the new "Owner account" field on
the edit forms.

See DECISIONS.md and HOW-IT-WORKS.md's "Accounts and roles" section for
the full reasoning and day-to-day behavior.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/laptop_register.xlsx
+++ b/laptop_register.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resignation" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Laptops'!$A$1:$R$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Laptops'!$A$1:$R$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Resignation'!$A$1:$H$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R8"/>
+  <dimension ref="A1:R10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -556,32 +556,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>نهي عبدالرازق احمد</t>
+          <t>مهند حماده جنش</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Noha Abdelrazek Ahmed</t>
+          <t>Mohannad Hamada Ganash</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1357</t>
+          <t>1355</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>nabdelrazek@stm.com.eg</t>
+          <t>mhamada@stm.com.eg</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>SLNAbdelrazekR</t>
+          <t>ITMHamadaR</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -591,7 +591,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>PF5T92HE</t>
+          <t>PF5NBNBH</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -640,17 +640,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>عمر اشرف احمد حبيب</t>
+          <t>سارة نبيل جورجي جرجس</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Omar Ashraf Ahmed Habib</t>
+          <t>Sara Nabil Gorgy Girgis</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1352</t>
+          <t>1353</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -660,12 +660,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ohabib@stm.com.eg</t>
+          <t>sanabil@stm.com.eg</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>SLOHabibR</t>
+          <t>SLSAnabilR</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -675,12 +675,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>PF5LX0S6</t>
+          <t>PF5NDMEY</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>I7</t>
+          <t>U5</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -705,12 +705,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>16-Sep-26</t>
+          <t>17-Sep-26</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Mohamed Taha</t>
+          <t>Majad</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -724,17 +724,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>مروة طارق احمد صبحي</t>
+          <t>نهي عبدالرازق احمد</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Marwa Tarek Ahmed Sobhy</t>
+          <t>Noha Abdelrazek Ahmed</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1351</t>
+          <t>1357</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -744,12 +744,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>matarek@stm.com.eg</t>
+          <t>nabdelrazek@stm.com.eg</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>SLMAtarekR</t>
+          <t>SLNAbdelrazekR</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -759,12 +759,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>PF5P93DS</t>
+          <t>PF5T92HE</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>U7</t>
+          <t>U5</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -789,12 +789,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>16-Sep-26</t>
+          <t>17-Sep-26</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Majad</t>
+          <t>Mohamed Taha</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -808,17 +808,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>فيصل هاني امام</t>
+          <t>عمر اشرف احمد حبيب</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Faisal hany Emam</t>
+          <t>Omar Ashraf Ahmed Habib</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1354</t>
+          <t>1352</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -828,12 +828,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>femam@stm.com.eg</t>
+          <t>ohabib@stm.com.eg</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>SLFEmamR</t>
+          <t>SLOHabibR</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -843,12 +843,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>PF5NG1YN</t>
+          <t>PF5LX0S6</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>I5</t>
+          <t>I7</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -892,32 +892,32 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>خالد عبد الخالق عبد المحسن</t>
+          <t>مروة طارق احمد صبحي</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Khaled Abdelkhalek Abdelmohsen</t>
+          <t>Marwa Tarek Ahmed Sobhy</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1350</t>
+          <t>1351</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>FM</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>kelsabahy@stm.com.eg</t>
+          <t>matarek@stm.com.eg</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>FMKElsabahyR</t>
+          <t>SLMAtarekR</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -927,12 +927,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>PF5W5TXH</t>
+          <t>PF5P93DS</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>I7</t>
+          <t>U7</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Mohamed Taha</t>
+          <t>Majad</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -976,47 +976,47 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>احمد ابراهيم صدقي</t>
+          <t>فيصل هاني امام</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ahmed Ibrahim Sedky</t>
+          <t>Faisal hany Emam</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1349</t>
+          <t>1354</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Administration</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>asedky@stm.com.eg</t>
+          <t>femam@stm.com.eg</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>ADASedkyR</t>
+          <t>SLFEmamR</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>E14</t>
+          <t>E16</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>PF5MDKBP</t>
+          <t>PF5NG1YN</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>I7</t>
+          <t>I5</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1060,47 +1060,47 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>محمد شعبان ابراهيم</t>
+          <t>خالد عبد الخالق عبد المحسن</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Mohamed Shaban Ibrahim</t>
+          <t>Khaled Abdelkhalek Abdelmohsen</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1356</t>
+          <t>1350</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>FM</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>mshaban@stm.com.eg</t>
+          <t>kelsabahy@stm.com.eg</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>SLMShabanR</t>
+          <t>FMKElsabahyR</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>E14</t>
+          <t>E16</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>PF5MG6KD</t>
+          <t>PF5W5TXH</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>U5</t>
+          <t>I7</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1141,8 +1141,176 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>احمد ابراهيم صدقي</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Ahmed Ibrahim Sedky</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1349</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>asedky@stm.com.eg</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>ADASedkyR</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>E14</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>PF5MDKBP</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>I7</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>24GB</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>512SSD</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>BLACK</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Laptop handover</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>16-Sep-26</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Mohamed Taha</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>Held</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>محمد شعبان ابراهيم</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Mohamed Shaban Ibrahim</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1356</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>mshaban@stm.com.eg</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>SLMShabanR</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>E14</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>PF5MG6KD</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>U5</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>24GB</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>512SSD</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>BLACK</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Laptop handover</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>16-Sep-26</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Mohamed Taha</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>Held</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R8"/>
+  <autoFilter ref="A1:R10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>